<commit_message>
Update person_class.py to correct template file reference and enhance order creation logic
</commit_message>
<xml_diff>
--- a/info.xlsx
+++ b/info.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="9" documentId="8_{3EACB3B8-4A11-4AF4-B688-D8FF6948FA02}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8EBDE894-AFC7-4B66-A298-57DBF5EE68DD}"/>
   <bookViews>
-    <workbookView xWindow="6225" yWindow="5295" windowWidth="28800" windowHeight="15345" xr2:uid="{5BA4D96A-8510-4D5D-90AD-627BFEDDF034}"/>
+    <workbookView xWindow="4680" yWindow="4680" windowWidth="28800" windowHeight="15345" xr2:uid="{5BA4D96A-8510-4D5D-90AD-627BFEDDF034}"/>
   </bookViews>
   <sheets>
     <sheet name="Ark1" sheetId="1" r:id="rId1"/>

</xml_diff>